<commit_message>
Case1 revalidated with final code
</commit_message>
<xml_diff>
--- a/01_Validasyon/Case1/time_alpha.xlsx
+++ b/01_Validasyon/Case1/time_alpha.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\barankucukcay\Desktop\Ablation-Modeling\01_Validasyon\Case1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6432B43-438E-4323-B3F8-7A39D1691487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D490F236-E84C-476F-B991-A3B736693466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -402,63 +402,48 @@
                   <c:v>81</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>82</c:v>
+                  <c:v>85</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>83</c:v>
+                  <c:v>87</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>84</c:v>
+                  <c:v>88</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>85</c:v>
+                  <c:v>89</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>86</c:v>
+                  <c:v>90</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>87</c:v>
+                  <c:v>91</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>88</c:v>
+                  <c:v>92</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>89</c:v>
+                  <c:v>93</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>90</c:v>
+                  <c:v>94</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>91</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>92</c:v>
+                  <c:v>96</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>93</c:v>
+                  <c:v>97</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>94</c:v>
+                  <c:v>98</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>95</c:v>
+                  <c:v>99</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>96</c:v>
-                </c:pt>
-                <c:pt idx="96">
-                  <c:v>97</c:v>
-                </c:pt>
-                <c:pt idx="97">
-                  <c:v>98</c:v>
-                </c:pt>
-                <c:pt idx="98">
-                  <c:v>99</c:v>
-                </c:pt>
-                <c:pt idx="99">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="100">
                   <c:v>100</c:v>
                 </c:pt>
               </c:numCache>
@@ -714,64 +699,49 @@
                   <c:v>0.92610000000000003</c:v>
                 </c:pt>
                 <c:pt idx="81">
-                  <c:v>0.92649999999999999</c:v>
+                  <c:v>0.92779999999999996</c:v>
                 </c:pt>
                 <c:pt idx="82">
-                  <c:v>0.92700000000000005</c:v>
+                  <c:v>0.92869999999999997</c:v>
                 </c:pt>
                 <c:pt idx="83">
-                  <c:v>0.9274</c:v>
+                  <c:v>0.92910000000000004</c:v>
                 </c:pt>
                 <c:pt idx="84">
-                  <c:v>0.92779999999999996</c:v>
+                  <c:v>0.92949999999999999</c:v>
                 </c:pt>
                 <c:pt idx="85">
-                  <c:v>0.92820000000000003</c:v>
+                  <c:v>0.92979999999999996</c:v>
                 </c:pt>
                 <c:pt idx="86">
-                  <c:v>0.92869999999999997</c:v>
+                  <c:v>0.93020000000000003</c:v>
                 </c:pt>
                 <c:pt idx="87">
-                  <c:v>0.92910000000000004</c:v>
+                  <c:v>0.93059999999999998</c:v>
                 </c:pt>
                 <c:pt idx="88">
-                  <c:v>0.92949999999999999</c:v>
+                  <c:v>0.93100000000000005</c:v>
                 </c:pt>
                 <c:pt idx="89">
-                  <c:v>0.92979999999999996</c:v>
+                  <c:v>0.93130000000000002</c:v>
                 </c:pt>
                 <c:pt idx="90">
-                  <c:v>0.93020000000000003</c:v>
+                  <c:v>0.93169999999999997</c:v>
                 </c:pt>
                 <c:pt idx="91">
-                  <c:v>0.93059999999999998</c:v>
+                  <c:v>0.93210000000000004</c:v>
                 </c:pt>
                 <c:pt idx="92">
-                  <c:v>0.93100000000000005</c:v>
+                  <c:v>0.93240000000000001</c:v>
                 </c:pt>
                 <c:pt idx="93">
-                  <c:v>0.93130000000000002</c:v>
+                  <c:v>0.93279999999999996</c:v>
                 </c:pt>
                 <c:pt idx="94">
-                  <c:v>0.93169999999999997</c:v>
+                  <c:v>0.93310000000000004</c:v>
                 </c:pt>
                 <c:pt idx="95">
-                  <c:v>0.93210000000000004</c:v>
-                </c:pt>
-                <c:pt idx="96">
-                  <c:v>0.93240000000000001</c:v>
-                </c:pt>
-                <c:pt idx="97">
-                  <c:v>0.93279999999999996</c:v>
-                </c:pt>
-                <c:pt idx="98">
-                  <c:v>0.93310000000000004</c:v>
-                </c:pt>
-                <c:pt idx="99">
                   <c:v>0.93340000000000001</c:v>
-                </c:pt>
-                <c:pt idx="100">
-                  <c:v>0.94740000000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1501,7 +1471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:I103"/>
+  <dimension ref="B3:I98"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="3" spans="2:9" x14ac:dyDescent="0.3">
@@ -2364,162 +2334,122 @@
     </row>
     <row r="84" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H84">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I84">
-        <v>0.92649999999999999</v>
+        <v>0.92779999999999996</v>
       </c>
     </row>
     <row r="85" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H85">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="I85">
-        <v>0.92700000000000005</v>
+        <v>0.92869999999999997</v>
       </c>
     </row>
     <row r="86" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H86">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="I86">
-        <v>0.9274</v>
+        <v>0.92910000000000004</v>
       </c>
     </row>
     <row r="87" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H87">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="I87">
-        <v>0.92779999999999996</v>
+        <v>0.92949999999999999</v>
       </c>
     </row>
     <row r="88" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H88">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="I88">
-        <v>0.92820000000000003</v>
+        <v>0.92979999999999996</v>
       </c>
     </row>
     <row r="89" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H89">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="I89">
-        <v>0.92869999999999997</v>
+        <v>0.93020000000000003</v>
       </c>
     </row>
     <row r="90" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H90">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I90">
-        <v>0.92910000000000004</v>
+        <v>0.93059999999999998</v>
       </c>
     </row>
     <row r="91" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H91">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="I91">
-        <v>0.92949999999999999</v>
+        <v>0.93100000000000005</v>
       </c>
     </row>
     <row r="92" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H92">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="I92">
-        <v>0.92979999999999996</v>
+        <v>0.93130000000000002</v>
       </c>
     </row>
     <row r="93" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H93">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="I93">
-        <v>0.93020000000000003</v>
+        <v>0.93169999999999997</v>
       </c>
     </row>
     <row r="94" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H94">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="I94">
-        <v>0.93059999999999998</v>
+        <v>0.93210000000000004</v>
       </c>
     </row>
     <row r="95" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H95">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I95">
-        <v>0.93100000000000005</v>
+        <v>0.93240000000000001</v>
       </c>
     </row>
     <row r="96" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H96">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I96">
-        <v>0.93130000000000002</v>
+        <v>0.93279999999999996</v>
       </c>
     </row>
     <row r="97" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H97">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I97">
-        <v>0.93169999999999997</v>
+        <v>0.93310000000000004</v>
       </c>
     </row>
     <row r="98" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H98">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="I98">
-        <v>0.93210000000000004</v>
-      </c>
-    </row>
-    <row r="99" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H99">
-        <v>97</v>
-      </c>
-      <c r="I99">
-        <v>0.93240000000000001</v>
-      </c>
-    </row>
-    <row r="100" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H100">
-        <v>98</v>
-      </c>
-      <c r="I100">
-        <v>0.93279999999999996</v>
-      </c>
-    </row>
-    <row r="101" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H101">
-        <v>99</v>
-      </c>
-      <c r="I101">
-        <v>0.93310000000000004</v>
-      </c>
-    </row>
-    <row r="102" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H102">
-        <v>100</v>
-      </c>
-      <c r="I102">
         <v>0.93340000000000001</v>
-      </c>
-    </row>
-    <row r="103" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H103">
-        <v>100</v>
-      </c>
-      <c r="I103">
-        <v>0.94740000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>